<commit_message>
Remove terminated employee Zhengjie Guan (237)
</commit_message>
<xml_diff>
--- a/employees_CA.xlsx
+++ b/employees_CA.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="164">
   <si>
     <t>Legal Name</t>
   </si>
@@ -106,9 +106,6 @@
     <t>Aixin</t>
   </si>
   <si>
-    <t>Zhengjie</t>
-  </si>
-  <si>
     <t>Bin</t>
   </si>
   <si>
@@ -332,9 +329,6 @@
   </si>
   <si>
     <t>Gu</t>
-  </si>
-  <si>
-    <t>Guan</t>
   </si>
   <si>
     <t>Guo</t>
@@ -847,7 +841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -896,22 +890,22 @@
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G2" s="1">
         <v>45916</v>
       </c>
       <c r="H2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I2" t="s">
         <v>148</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>150</v>
-      </c>
-      <c r="J2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -928,22 +922,22 @@
         <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G3" s="1">
         <v>46230</v>
       </c>
       <c r="H3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I3" t="s">
+        <v>149</v>
+      </c>
+      <c r="J3" t="s">
         <v>151</v>
-      </c>
-      <c r="J3" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -960,22 +954,22 @@
         <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G4" s="1">
         <v>44929</v>
       </c>
       <c r="H4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -992,22 +986,22 @@
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G5" s="1">
         <v>46168</v>
       </c>
       <c r="H5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1024,22 +1018,22 @@
         <v>17</v>
       </c>
       <c r="E6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G6" s="1">
         <v>43405</v>
       </c>
       <c r="H6" t="s">
+        <v>146</v>
+      </c>
+      <c r="I6" t="s">
         <v>148</v>
       </c>
-      <c r="I6" t="s">
-        <v>150</v>
-      </c>
       <c r="J6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -1056,22 +1050,22 @@
         <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G7" s="1">
         <v>45684</v>
       </c>
       <c r="H7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1088,22 +1082,22 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G8" s="1">
         <v>46223</v>
       </c>
       <c r="H8" t="s">
+        <v>146</v>
+      </c>
+      <c r="I8" t="s">
         <v>148</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>150</v>
-      </c>
-      <c r="J8" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1120,22 +1114,22 @@
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G9" s="1">
         <v>45909</v>
       </c>
       <c r="H9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I9" t="s">
+        <v>149</v>
+      </c>
+      <c r="J9" t="s">
         <v>151</v>
-      </c>
-      <c r="J9" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1152,22 +1146,22 @@
         <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G10" s="1">
         <v>45471</v>
       </c>
       <c r="H10" t="s">
+        <v>146</v>
+      </c>
+      <c r="I10" t="s">
         <v>148</v>
       </c>
-      <c r="I10" t="s">
-        <v>150</v>
-      </c>
       <c r="J10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1184,22 +1178,22 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F11" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G11" s="1">
         <v>45701</v>
       </c>
       <c r="H11" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I11" t="s">
+        <v>149</v>
+      </c>
+      <c r="J11" t="s">
         <v>151</v>
-      </c>
-      <c r="J11" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1216,22 +1210,22 @@
         <v>23</v>
       </c>
       <c r="E12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G12" s="1">
         <v>46225</v>
       </c>
       <c r="H12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1248,22 +1242,22 @@
         <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G13" s="1">
         <v>45538</v>
       </c>
       <c r="H13" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I13" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J13" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -1280,22 +1274,22 @@
         <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G14" s="1">
         <v>45915</v>
       </c>
       <c r="H14" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I14" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1312,22 +1306,22 @@
         <v>26</v>
       </c>
       <c r="E15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G15" s="1">
         <v>44317</v>
       </c>
       <c r="H15" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J15" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1344,22 +1338,22 @@
         <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F16" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G16" s="1">
         <v>45419</v>
       </c>
       <c r="H16" t="s">
+        <v>146</v>
+      </c>
+      <c r="I16" t="s">
         <v>148</v>
       </c>
-      <c r="I16" t="s">
-        <v>150</v>
-      </c>
       <c r="J16" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1376,22 +1370,22 @@
         <v>28</v>
       </c>
       <c r="E17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G17" s="1">
         <v>44069</v>
       </c>
       <c r="H17" t="s">
+        <v>146</v>
+      </c>
+      <c r="I17" t="s">
         <v>148</v>
       </c>
-      <c r="I17" t="s">
-        <v>150</v>
-      </c>
       <c r="J17" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1408,22 +1402,22 @@
         <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F18" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G18" s="1">
         <v>44756</v>
       </c>
       <c r="H18" t="s">
+        <v>146</v>
+      </c>
+      <c r="I18" t="s">
         <v>148</v>
       </c>
-      <c r="I18" t="s">
-        <v>150</v>
-      </c>
       <c r="J18" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1434,25 +1428,25 @@
         <v>12</v>
       </c>
       <c r="C19">
-        <v>237</v>
+        <v>2</v>
       </c>
       <c r="D19" t="s">
         <v>30</v>
       </c>
       <c r="E19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G19" s="1">
-        <v>46252</v>
+        <v>44348</v>
       </c>
       <c r="H19" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I19" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J19" t="s">
         <v>159</v>
@@ -1466,28 +1460,28 @@
         <v>12</v>
       </c>
       <c r="C20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="s">
         <v>31</v>
       </c>
       <c r="E20" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F20" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G20" s="1">
-        <v>44348</v>
+        <v>44452</v>
       </c>
       <c r="H20" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I20" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J20" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1498,28 +1492,28 @@
         <v>12</v>
       </c>
       <c r="C21">
-        <v>4</v>
+        <v>160</v>
       </c>
       <c r="D21" t="s">
         <v>32</v>
       </c>
       <c r="E21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F21" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G21" s="1">
-        <v>44452</v>
+        <v>45536</v>
       </c>
       <c r="H21" t="s">
+        <v>146</v>
+      </c>
+      <c r="I21" t="s">
         <v>148</v>
       </c>
-      <c r="I21" t="s">
-        <v>151</v>
-      </c>
       <c r="J21" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1530,28 +1524,28 @@
         <v>12</v>
       </c>
       <c r="C22">
-        <v>160</v>
+        <v>38</v>
       </c>
       <c r="D22" t="s">
         <v>33</v>
       </c>
       <c r="E22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F22" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G22" s="1">
-        <v>45536</v>
+        <v>44774</v>
       </c>
       <c r="H22" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I22" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J22" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1562,28 +1556,28 @@
         <v>12</v>
       </c>
       <c r="C23">
-        <v>38</v>
+        <v>225</v>
       </c>
       <c r="D23" t="s">
         <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F23" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G23" s="1">
-        <v>44774</v>
+        <v>46181</v>
       </c>
       <c r="H23" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I23" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J23" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -1594,28 +1588,28 @@
         <v>12</v>
       </c>
       <c r="C24">
-        <v>225</v>
+        <v>7</v>
       </c>
       <c r="D24" t="s">
         <v>35</v>
       </c>
       <c r="E24" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F24" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G24" s="1">
-        <v>46181</v>
+        <v>43564</v>
       </c>
       <c r="H24" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I24" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J24" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1626,92 +1620,92 @@
         <v>12</v>
       </c>
       <c r="C25">
-        <v>7</v>
+        <v>56</v>
       </c>
       <c r="D25" t="s">
         <v>36</v>
       </c>
       <c r="E25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F25" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G25" s="1">
-        <v>43564</v>
+        <v>44508</v>
       </c>
       <c r="H25" t="s">
+        <v>146</v>
+      </c>
+      <c r="I25" t="s">
         <v>148</v>
       </c>
-      <c r="I25" t="s">
-        <v>151</v>
-      </c>
       <c r="J25" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B26" t="s">
         <v>12</v>
       </c>
       <c r="C26">
-        <v>56</v>
+        <v>1044</v>
       </c>
       <c r="D26" t="s">
         <v>37</v>
       </c>
       <c r="E26" t="s">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="F26" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G26" s="1">
-        <v>44508</v>
+        <v>45689</v>
       </c>
       <c r="H26" t="s">
+        <v>146</v>
+      </c>
+      <c r="I26" t="s">
         <v>148</v>
       </c>
-      <c r="I26" t="s">
-        <v>150</v>
-      </c>
       <c r="J26" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
       </c>
       <c r="C27">
-        <v>1044</v>
+        <v>60</v>
       </c>
       <c r="D27" t="s">
         <v>38</v>
       </c>
       <c r="E27" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="F27" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G27" s="1">
-        <v>45689</v>
+        <v>44774</v>
       </c>
       <c r="H27" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I27" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J27" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -1722,28 +1716,28 @@
         <v>12</v>
       </c>
       <c r="C28">
-        <v>60</v>
+        <v>190</v>
       </c>
       <c r="D28" t="s">
         <v>39</v>
       </c>
       <c r="E28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F28" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G28" s="1">
-        <v>44774</v>
+        <v>45902</v>
       </c>
       <c r="H28" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I28" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J28" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -1754,28 +1748,28 @@
         <v>12</v>
       </c>
       <c r="C29">
-        <v>190</v>
+        <v>77</v>
       </c>
       <c r="D29" t="s">
         <v>40</v>
       </c>
       <c r="E29" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F29" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G29" s="1">
-        <v>45902</v>
+        <v>45047</v>
       </c>
       <c r="H29" t="s">
+        <v>146</v>
+      </c>
+      <c r="I29" t="s">
         <v>148</v>
       </c>
-      <c r="I29" t="s">
-        <v>151</v>
-      </c>
       <c r="J29" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -1786,28 +1780,28 @@
         <v>12</v>
       </c>
       <c r="C30">
-        <v>77</v>
+        <v>182</v>
       </c>
       <c r="D30" t="s">
         <v>41</v>
       </c>
       <c r="E30" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F30" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G30" s="1">
-        <v>45047</v>
+        <v>45859</v>
       </c>
       <c r="H30" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I30" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J30" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -1818,28 +1812,28 @@
         <v>12</v>
       </c>
       <c r="C31">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D31" t="s">
         <v>42</v>
       </c>
       <c r="E31" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F31" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G31" s="1">
         <v>45859</v>
       </c>
       <c r="H31" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I31" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J31" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -1850,28 +1844,28 @@
         <v>12</v>
       </c>
       <c r="C32">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D32" t="s">
         <v>43</v>
       </c>
       <c r="E32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F32" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G32" s="1">
-        <v>45859</v>
+        <v>45809</v>
       </c>
       <c r="H32" t="s">
+        <v>146</v>
+      </c>
+      <c r="I32" t="s">
         <v>148</v>
       </c>
-      <c r="I32" t="s">
-        <v>151</v>
-      </c>
       <c r="J32" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1882,28 +1876,28 @@
         <v>12</v>
       </c>
       <c r="C33">
-        <v>177</v>
+        <v>208</v>
       </c>
       <c r="D33" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E33" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F33" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G33" s="1">
-        <v>45809</v>
+        <v>46017</v>
       </c>
       <c r="H33" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I33" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J33" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -1914,28 +1908,28 @@
         <v>12</v>
       </c>
       <c r="C34">
-        <v>208</v>
+        <v>5</v>
       </c>
       <c r="D34" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G34" s="1">
-        <v>46017</v>
+        <v>45313</v>
       </c>
       <c r="H34" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I34" t="s">
+        <v>149</v>
+      </c>
+      <c r="J34" t="s">
         <v>151</v>
-      </c>
-      <c r="J34" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -1946,28 +1940,28 @@
         <v>12</v>
       </c>
       <c r="C35">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="D35" t="s">
         <v>45</v>
       </c>
       <c r="E35" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F35" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G35" s="1">
-        <v>45313</v>
+        <v>44858</v>
       </c>
       <c r="H35" t="s">
+        <v>146</v>
+      </c>
+      <c r="I35" t="s">
         <v>148</v>
       </c>
-      <c r="I35" t="s">
-        <v>151</v>
-      </c>
       <c r="J35" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -1978,28 +1972,28 @@
         <v>12</v>
       </c>
       <c r="C36">
-        <v>58</v>
+        <v>169</v>
       </c>
       <c r="D36" t="s">
         <v>46</v>
       </c>
       <c r="E36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F36" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G36" s="1">
-        <v>44858</v>
+        <v>45600</v>
       </c>
       <c r="H36" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I36" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J36" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -2010,25 +2004,25 @@
         <v>12</v>
       </c>
       <c r="C37">
-        <v>169</v>
+        <v>207</v>
       </c>
       <c r="D37" t="s">
         <v>47</v>
       </c>
       <c r="E37" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F37" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G37" s="1">
-        <v>45600</v>
+        <v>46197</v>
       </c>
       <c r="H37" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I37" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J37" t="s">
         <v>153</v>
@@ -2042,28 +2036,28 @@
         <v>12</v>
       </c>
       <c r="C38">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D38" t="s">
         <v>48</v>
       </c>
       <c r="E38" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F38" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G38" s="1">
-        <v>46197</v>
+        <v>46113</v>
       </c>
       <c r="H38" t="s">
+        <v>146</v>
+      </c>
+      <c r="I38" t="s">
         <v>148</v>
       </c>
-      <c r="I38" t="s">
-        <v>151</v>
-      </c>
       <c r="J38" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -2074,28 +2068,28 @@
         <v>12</v>
       </c>
       <c r="C39">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D39" t="s">
         <v>49</v>
       </c>
       <c r="E39" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F39" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G39" s="1">
-        <v>46113</v>
+        <v>46070</v>
       </c>
       <c r="H39" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I39" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J39" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -2106,28 +2100,28 @@
         <v>12</v>
       </c>
       <c r="C40">
-        <v>212</v>
+        <v>238</v>
       </c>
       <c r="D40" t="s">
         <v>50</v>
       </c>
       <c r="E40" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F40" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G40" s="1">
-        <v>46070</v>
+        <v>46254</v>
       </c>
       <c r="H40" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I40" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J40" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -2138,25 +2132,25 @@
         <v>12</v>
       </c>
       <c r="C41">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D41" t="s">
         <v>51</v>
       </c>
       <c r="E41" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F41" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G41" s="1">
-        <v>46254</v>
+        <v>46181</v>
       </c>
       <c r="H41" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I41" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J41" t="s">
         <v>155</v>
@@ -2170,28 +2164,28 @@
         <v>12</v>
       </c>
       <c r="C42">
-        <v>226</v>
+        <v>48</v>
       </c>
       <c r="D42" t="s">
         <v>52</v>
       </c>
       <c r="E42" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F42" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G42" s="1">
-        <v>46181</v>
+        <v>44348</v>
       </c>
       <c r="H42" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I42" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J42" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -2202,28 +2196,28 @@
         <v>12</v>
       </c>
       <c r="C43">
-        <v>48</v>
+        <v>122</v>
       </c>
       <c r="D43" t="s">
         <v>53</v>
       </c>
       <c r="E43" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F43" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G43" s="1">
-        <v>44348</v>
+        <v>46126</v>
       </c>
       <c r="H43" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I43" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J43" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -2234,28 +2228,28 @@
         <v>12</v>
       </c>
       <c r="C44">
-        <v>122</v>
+        <v>46</v>
       </c>
       <c r="D44" t="s">
         <v>54</v>
       </c>
       <c r="E44" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F44" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G44" s="1">
-        <v>46126</v>
+        <v>44802</v>
       </c>
       <c r="H44" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I44" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J44" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -2266,28 +2260,28 @@
         <v>12</v>
       </c>
       <c r="C45">
-        <v>46</v>
+        <v>234</v>
       </c>
       <c r="D45" t="s">
         <v>55</v>
       </c>
       <c r="E45" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F45" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G45" s="1">
-        <v>44802</v>
+        <v>46237</v>
       </c>
       <c r="H45" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I45" t="s">
+        <v>149</v>
+      </c>
+      <c r="J45" t="s">
         <v>151</v>
-      </c>
-      <c r="J45" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -2298,28 +2292,28 @@
         <v>12</v>
       </c>
       <c r="C46">
-        <v>234</v>
+        <v>141</v>
       </c>
       <c r="D46" t="s">
         <v>56</v>
       </c>
       <c r="E46" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F46" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G46" s="1">
-        <v>46237</v>
+        <v>45499</v>
       </c>
       <c r="H46" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I46" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J46" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -2330,28 +2324,28 @@
         <v>12</v>
       </c>
       <c r="C47">
-        <v>141</v>
+        <v>200</v>
       </c>
       <c r="D47" t="s">
         <v>57</v>
       </c>
       <c r="E47" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F47" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G47" s="1">
-        <v>45499</v>
+        <v>45957</v>
       </c>
       <c r="H47" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I47" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J47" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" spans="1:10">
@@ -2362,28 +2356,28 @@
         <v>12</v>
       </c>
       <c r="C48">
-        <v>200</v>
+        <v>15</v>
       </c>
       <c r="D48" t="s">
         <v>58</v>
       </c>
       <c r="E48" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F48" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G48" s="1">
-        <v>45957</v>
+        <v>43922</v>
       </c>
       <c r="H48" t="s">
+        <v>146</v>
+      </c>
+      <c r="I48" t="s">
         <v>148</v>
       </c>
-      <c r="I48" t="s">
-        <v>151</v>
-      </c>
       <c r="J48" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -2394,28 +2388,28 @@
         <v>12</v>
       </c>
       <c r="C49">
-        <v>15</v>
+        <v>165</v>
       </c>
       <c r="D49" t="s">
         <v>59</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F49" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G49" s="1">
-        <v>43922</v>
+        <v>45579</v>
       </c>
       <c r="H49" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I49" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J49" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -2426,28 +2420,28 @@
         <v>12</v>
       </c>
       <c r="C50">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
         <v>60</v>
       </c>
       <c r="E50" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F50" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G50" s="1">
-        <v>45579</v>
+        <v>45509</v>
       </c>
       <c r="H50" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I50" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J50" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -2458,156 +2452,156 @@
         <v>12</v>
       </c>
       <c r="C51">
-        <v>147</v>
+        <v>235</v>
       </c>
       <c r="D51" t="s">
         <v>61</v>
       </c>
       <c r="E51" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F51" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G51" s="1">
-        <v>45509</v>
+        <v>46244</v>
       </c>
       <c r="H51" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I51" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J51" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
         <v>12</v>
       </c>
       <c r="C52">
-        <v>235</v>
+        <v>1028</v>
       </c>
       <c r="D52" t="s">
         <v>62</v>
       </c>
       <c r="E52" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F52" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G52" s="1">
-        <v>46244</v>
+        <v>45239</v>
       </c>
       <c r="H52" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I52" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J52" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B53" t="s">
         <v>12</v>
       </c>
       <c r="C53">
-        <v>1028</v>
+        <v>85</v>
       </c>
       <c r="D53" t="s">
         <v>63</v>
       </c>
       <c r="E53" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F53" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G53" s="1">
-        <v>45239</v>
+        <v>46181</v>
       </c>
       <c r="H53" t="s">
+        <v>146</v>
+      </c>
+      <c r="I53" t="s">
         <v>148</v>
       </c>
-      <c r="I53" t="s">
-        <v>151</v>
-      </c>
       <c r="J53" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
         <v>12</v>
       </c>
       <c r="C54">
-        <v>85</v>
+        <v>1043</v>
       </c>
       <c r="D54" t="s">
         <v>64</v>
       </c>
       <c r="E54" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F54" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G54" s="1">
-        <v>46181</v>
+        <v>45680</v>
       </c>
       <c r="H54" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I54" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J54" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B55" t="s">
         <v>12</v>
       </c>
       <c r="C55">
-        <v>1043</v>
+        <v>218</v>
       </c>
       <c r="D55" t="s">
         <v>65</v>
       </c>
       <c r="E55" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F55" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G55" s="1">
-        <v>45680</v>
+        <v>46127</v>
       </c>
       <c r="H55" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I55" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J55" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -2618,28 +2612,28 @@
         <v>12</v>
       </c>
       <c r="C56">
-        <v>218</v>
+        <v>176</v>
       </c>
       <c r="D56" t="s">
         <v>66</v>
       </c>
       <c r="E56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F56" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G56" s="1">
-        <v>46127</v>
+        <v>45778</v>
       </c>
       <c r="H56" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I56" t="s">
+        <v>149</v>
+      </c>
+      <c r="J56" t="s">
         <v>151</v>
-      </c>
-      <c r="J56" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -2650,28 +2644,28 @@
         <v>12</v>
       </c>
       <c r="C57">
-        <v>176</v>
+        <v>41</v>
       </c>
       <c r="D57" t="s">
         <v>67</v>
       </c>
       <c r="E57" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F57" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G57" s="1">
-        <v>45778</v>
+        <v>44537</v>
       </c>
       <c r="H57" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I57" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J57" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -2682,220 +2676,220 @@
         <v>12</v>
       </c>
       <c r="C58">
-        <v>41</v>
+        <v>233</v>
       </c>
       <c r="D58" t="s">
         <v>68</v>
       </c>
       <c r="E58" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F58" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G58" s="1">
-        <v>44537</v>
+        <v>46237</v>
       </c>
       <c r="H58" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I58" t="s">
+        <v>149</v>
+      </c>
+      <c r="J58" t="s">
         <v>151</v>
-      </c>
-      <c r="J58" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
         <v>12</v>
       </c>
       <c r="C59">
-        <v>233</v>
+        <v>1017</v>
       </c>
       <c r="D59" t="s">
         <v>69</v>
       </c>
       <c r="E59" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F59" t="s">
+        <v>145</v>
+      </c>
+      <c r="G59" s="1">
+        <v>45062</v>
+      </c>
+      <c r="H59" t="s">
         <v>147</v>
       </c>
-      <c r="G59" s="1">
-        <v>46237</v>
-      </c>
-      <c r="H59" t="s">
+      <c r="I59" t="s">
         <v>148</v>
       </c>
-      <c r="I59" t="s">
-        <v>151</v>
-      </c>
       <c r="J59" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B60" t="s">
         <v>12</v>
       </c>
       <c r="C60">
-        <v>1017</v>
+        <v>166</v>
       </c>
       <c r="D60" t="s">
         <v>70</v>
       </c>
       <c r="E60" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F60" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G60" s="1">
-        <v>45062</v>
+        <v>45586</v>
       </c>
       <c r="H60" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I60" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J60" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
         <v>12</v>
       </c>
       <c r="C61">
-        <v>166</v>
+        <v>1041</v>
       </c>
       <c r="D61" t="s">
         <v>71</v>
       </c>
       <c r="E61" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F61" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G61" s="1">
-        <v>45586</v>
+        <v>45689</v>
       </c>
       <c r="H61" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I61" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J61" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B62" t="s">
         <v>12</v>
       </c>
       <c r="C62">
-        <v>1041</v>
+        <v>209</v>
       </c>
       <c r="D62" t="s">
         <v>72</v>
       </c>
       <c r="E62" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F62" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G62" s="1">
-        <v>45689</v>
+        <v>46048</v>
       </c>
       <c r="H62" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I62" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J62" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B63" t="s">
         <v>12</v>
       </c>
       <c r="C63">
-        <v>209</v>
+        <v>1027</v>
       </c>
       <c r="D63" t="s">
         <v>73</v>
       </c>
       <c r="E63" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F63" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G63" s="1">
-        <v>46048</v>
+        <v>45176</v>
       </c>
       <c r="H63" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I63" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J63" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B64" t="s">
         <v>12</v>
       </c>
       <c r="C64">
-        <v>1027</v>
+        <v>21</v>
       </c>
       <c r="D64" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E64" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F64" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G64" s="1">
-        <v>45176</v>
+        <v>45243</v>
       </c>
       <c r="H64" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I64" t="s">
+        <v>149</v>
+      </c>
+      <c r="J64" t="s">
         <v>151</v>
-      </c>
-      <c r="J64" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -2906,89 +2900,89 @@
         <v>12</v>
       </c>
       <c r="C65">
-        <v>21</v>
+        <v>220</v>
       </c>
       <c r="D65" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E65" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F65" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G65" s="1">
-        <v>45243</v>
+        <v>46141</v>
       </c>
       <c r="H65" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I65" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J65" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B66" t="s">
         <v>12</v>
       </c>
       <c r="C66">
-        <v>220</v>
+        <v>1013</v>
       </c>
       <c r="D66" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="E66" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G66" s="1">
-        <v>46141</v>
+        <v>44929</v>
       </c>
       <c r="H66" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I66" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J66" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B67" t="s">
         <v>12</v>
       </c>
       <c r="C67">
-        <v>1013</v>
+        <v>223</v>
       </c>
       <c r="D67" t="s">
         <v>75</v>
       </c>
       <c r="E67" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F67" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G67" s="1">
-        <v>44929</v>
+        <v>46163</v>
       </c>
       <c r="H67" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I67" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J67" t="s">
         <v>154</v>
@@ -3002,28 +2996,28 @@
         <v>12</v>
       </c>
       <c r="C68">
-        <v>223</v>
+        <v>121</v>
       </c>
       <c r="D68" t="s">
         <v>76</v>
       </c>
       <c r="E68" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F68" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G68" s="1">
-        <v>46163</v>
+        <v>45432</v>
       </c>
       <c r="H68" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I68" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J68" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -3034,28 +3028,28 @@
         <v>12</v>
       </c>
       <c r="C69">
-        <v>121</v>
+        <v>65</v>
       </c>
       <c r="D69" t="s">
         <v>77</v>
       </c>
       <c r="E69" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F69" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G69" s="1">
-        <v>45432</v>
+        <v>44909</v>
       </c>
       <c r="H69" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I69" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J69" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -3066,28 +3060,28 @@
         <v>12</v>
       </c>
       <c r="C70">
-        <v>65</v>
+        <v>205</v>
       </c>
       <c r="D70" t="s">
         <v>78</v>
       </c>
       <c r="E70" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F70" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G70" s="1">
-        <v>44909</v>
+        <v>45978</v>
       </c>
       <c r="H70" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I70" t="s">
+        <v>149</v>
+      </c>
+      <c r="J70" t="s">
         <v>151</v>
-      </c>
-      <c r="J70" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="71" spans="1:10">
@@ -3098,28 +3092,28 @@
         <v>12</v>
       </c>
       <c r="C71">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D71" t="s">
         <v>79</v>
       </c>
       <c r="E71" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F71" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G71" s="1">
-        <v>45978</v>
+        <v>45938</v>
       </c>
       <c r="H71" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I71" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J71" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="72" spans="1:10">
@@ -3130,28 +3124,28 @@
         <v>12</v>
       </c>
       <c r="C72">
-        <v>199</v>
+        <v>221</v>
       </c>
       <c r="D72" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E72" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F72" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G72" s="1">
-        <v>45938</v>
+        <v>46146</v>
       </c>
       <c r="H72" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I72" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J72" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="73" spans="1:10">
@@ -3162,28 +3156,28 @@
         <v>12</v>
       </c>
       <c r="C73">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="D73" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="E73" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F73" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G73" s="1">
-        <v>46146</v>
+        <v>46076</v>
       </c>
       <c r="H73" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I73" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J73" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="74" spans="1:10">
@@ -3194,57 +3188,57 @@
         <v>12</v>
       </c>
       <c r="C74">
-        <v>213</v>
+        <v>127</v>
       </c>
       <c r="D74" t="s">
         <v>81</v>
       </c>
       <c r="E74" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F74" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G74" s="1">
-        <v>46076</v>
+        <v>45444</v>
       </c>
       <c r="H74" t="s">
+        <v>146</v>
+      </c>
+      <c r="I74" t="s">
         <v>148</v>
       </c>
-      <c r="I74" t="s">
-        <v>151</v>
-      </c>
       <c r="J74" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B75" t="s">
         <v>12</v>
       </c>
       <c r="C75">
-        <v>127</v>
+        <v>1008</v>
       </c>
       <c r="D75" t="s">
         <v>82</v>
       </c>
       <c r="E75" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F75" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G75" s="1">
-        <v>45444</v>
+        <v>46007</v>
       </c>
       <c r="H75" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I75" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J75" t="s">
         <v>152</v>
@@ -3252,34 +3246,34 @@
     </row>
     <row r="76" spans="1:10">
       <c r="A76" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B76" t="s">
         <v>12</v>
       </c>
       <c r="C76">
-        <v>1008</v>
+        <v>214</v>
       </c>
       <c r="D76" t="s">
         <v>83</v>
       </c>
       <c r="E76" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F76" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G76" s="1">
-        <v>46007</v>
+        <v>46076</v>
       </c>
       <c r="H76" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I76" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J76" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="77" spans="1:10">
@@ -3290,28 +3284,28 @@
         <v>12</v>
       </c>
       <c r="C77">
-        <v>214</v>
+        <v>189</v>
       </c>
       <c r="D77" t="s">
         <v>84</v>
       </c>
       <c r="E77" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F77" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G77" s="1">
-        <v>46076</v>
+        <v>45894</v>
       </c>
       <c r="H77" t="s">
+        <v>146</v>
+      </c>
+      <c r="I77" t="s">
         <v>148</v>
       </c>
-      <c r="I77" t="s">
-        <v>151</v>
-      </c>
       <c r="J77" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="78" spans="1:10">
@@ -3322,25 +3316,25 @@
         <v>12</v>
       </c>
       <c r="C78">
-        <v>189</v>
+        <v>9</v>
       </c>
       <c r="D78" t="s">
         <v>85</v>
       </c>
       <c r="E78" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F78" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G78" s="1">
-        <v>45894</v>
+        <v>44287</v>
       </c>
       <c r="H78" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J78" t="s">
         <v>159</v>
@@ -3354,28 +3348,28 @@
         <v>12</v>
       </c>
       <c r="C79">
-        <v>9</v>
+        <v>204</v>
       </c>
       <c r="D79" t="s">
         <v>86</v>
       </c>
       <c r="E79" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F79" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G79" s="1">
-        <v>44287</v>
+        <v>45978</v>
       </c>
       <c r="H79" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I79" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J79" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="80" spans="1:10">
@@ -3386,28 +3380,28 @@
         <v>12</v>
       </c>
       <c r="C80">
-        <v>204</v>
+        <v>22</v>
       </c>
       <c r="D80" t="s">
         <v>87</v>
       </c>
       <c r="E80" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F80" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G80" s="1">
-        <v>45978</v>
+        <v>44683</v>
       </c>
       <c r="H80" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I80" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J80" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="81" spans="1:10">
@@ -3418,28 +3412,28 @@
         <v>12</v>
       </c>
       <c r="C81">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="D81" t="s">
         <v>88</v>
       </c>
       <c r="E81" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F81" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G81" s="1">
-        <v>44683</v>
+        <v>46153</v>
       </c>
       <c r="H81" t="s">
+        <v>146</v>
+      </c>
+      <c r="I81" t="s">
         <v>148</v>
       </c>
-      <c r="I81" t="s">
-        <v>151</v>
-      </c>
       <c r="J81" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="82" spans="1:10">
@@ -3450,28 +3444,28 @@
         <v>12</v>
       </c>
       <c r="C82">
-        <v>228</v>
+        <v>187</v>
       </c>
       <c r="D82" t="s">
         <v>89</v>
       </c>
       <c r="E82" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F82" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G82" s="1">
-        <v>46153</v>
+        <v>45873</v>
       </c>
       <c r="H82" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I82" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J82" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
     </row>
     <row r="83" spans="1:10">
@@ -3482,25 +3476,25 @@
         <v>12</v>
       </c>
       <c r="C83">
-        <v>187</v>
+        <v>84</v>
       </c>
       <c r="D83" t="s">
         <v>90</v>
       </c>
       <c r="E83" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F83" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G83" s="1">
-        <v>45873</v>
+        <v>45121</v>
       </c>
       <c r="H83" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I83" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J83" t="s">
         <v>153</v>
@@ -3514,28 +3508,28 @@
         <v>12</v>
       </c>
       <c r="C84">
-        <v>84</v>
+        <v>198</v>
       </c>
       <c r="D84" t="s">
         <v>91</v>
       </c>
       <c r="E84" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F84" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G84" s="1">
-        <v>45121</v>
+        <v>45936</v>
       </c>
       <c r="H84" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I84" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J84" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="85" spans="1:10">
@@ -3546,28 +3540,28 @@
         <v>12</v>
       </c>
       <c r="C85">
-        <v>198</v>
+        <v>133</v>
       </c>
       <c r="D85" t="s">
         <v>92</v>
       </c>
       <c r="E85" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F85" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G85" s="1">
-        <v>45936</v>
+        <v>45957</v>
       </c>
       <c r="H85" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I85" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J85" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
     </row>
     <row r="86" spans="1:10">
@@ -3578,60 +3572,28 @@
         <v>12</v>
       </c>
       <c r="C86">
-        <v>133</v>
+        <v>3</v>
       </c>
       <c r="D86" t="s">
         <v>93</v>
       </c>
       <c r="E86" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F86" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G86" s="1">
-        <v>45957</v>
+        <v>44348</v>
       </c>
       <c r="H86" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I86" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J86" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10">
-      <c r="A87" t="s">
-        <v>10</v>
-      </c>
-      <c r="B87" t="s">
-        <v>12</v>
-      </c>
-      <c r="C87">
-        <v>3</v>
-      </c>
-      <c r="D87" t="s">
-        <v>94</v>
-      </c>
-      <c r="E87" t="s">
-        <v>146</v>
-      </c>
-      <c r="F87" t="s">
-        <v>147</v>
-      </c>
-      <c r="G87" s="1">
-        <v>44348</v>
-      </c>
-      <c r="H87" t="s">
-        <v>148</v>
-      </c>
-      <c r="I87" t="s">
-        <v>151</v>
-      </c>
-      <c r="J87" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>